<commit_message>
fix(productos): datos del manual — el retimbrado de extintores vence de verdad (2021-05-09 → próxima 2026-05-09): el calendario legal muestra 1 vencido, coherente con el plan de 90 días y el acuerdo A20
Via: Claude Code

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCSWTY9vg31r79SS3C87Rt
</commit_message>
<xml_diff>
--- a/scripts/productos-digitales/manual-manager/build/calendario-cumplimiento-legal.xlsx
+++ b/scripts/productos-digitales/manual-manager/build/calendario-cumplimiento-legal.xlsx
@@ -1616,7 +1616,7 @@
         </is>
       </c>
       <c r="C14" s="16" t="n">
-        <v>45055</v>
+        <v>44325</v>
       </c>
       <c r="D14" s="17" t="n">
         <v>60</v>
@@ -1628,15 +1628,15 @@
       </c>
       <c r="F14" s="11">
         <f>IFERROR(IF(OR($C14="",$D14=""),"",IF($D14=0,"",EDATE($C14,$D14))),"")</f>
-        <v>46882.0</v>
+        <v>46151.0</v>
       </c>
       <c r="G14" s="18">
         <f>IFERROR(IF(OR($F14="",$C$5=""),"",$F14-$C$5),"")</f>
-        <v>613.0</v>
+        <v>-118.0</v>
       </c>
       <c r="H14" s="12" t="str">
         <f>IFERROR(IF($B14="","",IF($D14=0,"No vence",IF($F14="","",IF($G14&lt;0,"VENCIDO",IF($G14&lt;=$C$6,"&lt; "&amp;TEXT($C$6,"0")&amp;" días",IF($G14&lt;=$C$7,"&lt; "&amp;TEXT($C$7,"0")&amp;" días","OK")))))),"")</f>
-        <v>OK</v>
+        <v>VENCIDO</v>
       </c>
       <c r="I14" s="12" t="inlineStr"/>
       <c r="J14" s="12" t="inlineStr"/>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="D43" s="20">
         <f>COUNTIF($G$10:$G$35,"&lt;0")</f>
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="44">
@@ -2594,7 +2594,7 @@
       </c>
       <c r="D46" s="9">
         <f>COUNTIFS($G$10:$G$35,"&gt;"&amp;$C$7)</f>
-        <v>13.0</v>
+        <v>12.0</v>
       </c>
     </row>
     <row r="47">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="D47" s="21">
         <f>IFERROR(IF($D$42=0,"",$D$46/$D$42),"")</f>
-        <v>0.8125</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="48"/>

</xml_diff>